<commit_message>
Fix bugs: dynamic XML row insertion, formula evaluated values, robust GST reconciliation, and clean register totals
</commit_message>
<xml_diff>
--- a/1. Expense_Invoice_Register.xlsx
+++ b/1. Expense_Invoice_Register.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns2="http://schemas.libreoffice.org/" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -13,12 +13,12 @@
     <sheet name="Emails Not Scanned" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Invoice Register'!$A$4:$AT$121</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Invoice Register'!$A$4:$AT$128</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    <ext uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <ns2:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -19257,37 +19257,43 @@
     </row>
     <row r="122" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="47" t="n">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B122" s="47" t="inlineStr">
         <is>
-          <t>IPinfo Inc\3MNDSIX0-0003 04.10.26.pdf</t>
+          <t>XTO10X Technologies Private Limited\2026-27-224 01.10.26.pdf</t>
         </is>
       </c>
       <c r="C122" s="47" t="inlineStr">
         <is>
-          <t>3MNDSIX0/0003</t>
+          <t>2026-27/224</t>
         </is>
       </c>
       <c r="D122" s="48" t="n">
-        <v>46299</v>
+        <v>46296</v>
       </c>
       <c r="E122" s="49" t="n">
         <f aca="false">YEAR(D122)</f>
+        <v>2026</v>
       </c>
       <c r="F122" s="50" t="str">
         <f aca="false">TEXT(D122,"mmm")</f>
+        <v>Oct</v>
       </c>
       <c r="G122" s="47" t="inlineStr">
         <is>
-          <t>IPinfo Inc</t>
+          <t>XTO10X Technologies Private Limited</t>
         </is>
       </c>
-      <c r="H122" s="47"/>
+      <c r="H122" s="47" t="inlineStr">
+        <is>
+          <t>29AAACX2697R1Z9</t>
+        </is>
+      </c>
       <c r="I122" s="47"/>
       <c r="J122" s="47" t="inlineStr">
         <is>
-          <t>Expense / Services - IPinfo Inc</t>
+          <t>XTO10X Technologies Private Limited - invoice 2026-27/224</t>
         </is>
       </c>
       <c r="K122" s="55"/>
@@ -19301,55 +19307,66 @@
         </is>
       </c>
       <c r="O122" s="51" t="n">
-        <v>0.0</v>
+        <v>1000000.0</v>
       </c>
       <c r="P122" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="Q122" s="52" t="n">
         <f aca="false">M122*O122-P122</f>
+        <v>1000000.0</v>
       </c>
       <c r="R122" s="53" t="n">
-        <v>0.0</v>
+        <v>0.18</v>
       </c>
       <c r="S122" s="47" t="inlineStr">
         <is>
-          <t>No GST (unregistered)</t>
+          <t>IGST</t>
         </is>
       </c>
       <c r="T122" s="52" t="n">
         <f aca="false">IF(S122="IGST",ROUND(Q122*R122,2),0)</f>
+        <v>180000.0</v>
       </c>
       <c r="U122" s="52" t="n">
         <f aca="false">IF(S122="CGST+SGST",ROUND(Q122*R122/2,2),0)</f>
+        <v>0.0</v>
       </c>
       <c r="V122" s="52" t="n">
         <f aca="false">U122</f>
+        <v>0.0</v>
       </c>
       <c r="W122" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="X122" s="52" t="n">
         <f aca="false">Q122+T122+U122+V122+W122</f>
+        <v>1180000.0</v>
       </c>
       <c r="Y122" s="52" t="n">
         <f aca="false">ROUND(Q122*AT122,0)</f>
+        <v>20000.0</v>
       </c>
       <c r="Z122" s="52" t="n">
         <f aca="false">X122-Y122</f>
+        <v>1160000.0</v>
       </c>
       <c r="AA122" s="47"/>
       <c r="AB122" s="47"/>
       <c r="AC122" s="47"/>
-      <c r="AD122" s="47"/>
+      <c r="AD122" s="47" t="inlineStr">
+        <is>
+          <t>Karnataka (29)</t>
+        </is>
+      </c>
       <c r="AE122" s="47" t="inlineStr">
         <is>
-          <t>06AAFCN6567R1ZL</t>
+          <t>07AAFCN6567R2ZI</t>
         </is>
       </c>
       <c r="AF122" s="47" t="inlineStr">
         <is>
-          <t>Haryana (06)</t>
+          <t>Delhi (07)</t>
         </is>
       </c>
       <c r="AG122" s="47"/>
@@ -19365,30 +19382,30 @@
       <c r="AQ122" s="47"/>
       <c r="AR122" s="47" t="inlineStr">
         <is>
-          <t>No RCM – forward charge; CGST + SGST charged by supplier. ITC eligible (check GSTR-2B).</t>
+          <t>No RCM - forward charge; IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
         </is>
       </c>
       <c r="AS122" s="47" t="inlineStr">
         <is>
-          <t>Sec 393(1) – purchase of goods (old 194Q), code 1031. Apply only if FY purchases from this supplier &gt; ₹50 L (on excess).</t>
+          <t>194J</t>
         </is>
       </c>
       <c r="AT122" s="54" t="n">
-        <v>0.001</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="47" t="n">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B123" s="47" t="inlineStr">
         <is>
-          <t>Mahindra &amp; Mahindra Financial Services Limited\231742 01.10.26.pdf</t>
+          <t>Mahindra &amp; Mahindra Financial Services Limited\IND-450459 01.10.26.pdf</t>
         </is>
       </c>
       <c r="C123" s="47" t="inlineStr">
         <is>
-          <t>231742</t>
+          <t>IND-450459</t>
         </is>
       </c>
       <c r="D123" s="48" t="n">
@@ -19396,9 +19413,11 @@
       </c>
       <c r="E123" s="49" t="n">
         <f aca="false">YEAR(D123)</f>
+        <v>2026</v>
       </c>
       <c r="F123" s="50" t="str">
         <f aca="false">TEXT(D123,"mmm")</f>
+        <v>Oct</v>
       </c>
       <c r="G123" s="47" t="inlineStr">
         <is>
@@ -19413,10 +19432,14 @@
       <c r="I123" s="47"/>
       <c r="J123" s="47" t="inlineStr">
         <is>
-          <t>Expense / Services - Mahindra &amp; Mahindra Financial Services Limited</t>
+          <t>Lease Rental - Kia Sonet 1.0 T-GDI HTX DCT Petrol _ HR26FR5339 110949-1 ARUN KUMAR PANIGRAHI NBE00141</t>
         </is>
       </c>
-      <c r="K123" s="55"/>
+      <c r="K123" s="55" t="inlineStr">
+        <is>
+          <t>997319</t>
+        </is>
+      </c>
       <c r="L123" s="47"/>
       <c r="M123" s="47" t="n">
         <v>1.0</v>
@@ -19427,13 +19450,14 @@
         </is>
       </c>
       <c r="O123" s="51" t="n">
-        <v>20506.19</v>
+        <v>44735.13</v>
       </c>
       <c r="P123" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="Q123" s="52" t="n">
         <f aca="false">M123*O123-P123</f>
+        <v>44735.13</v>
       </c>
       <c r="R123" s="53" t="n">
         <v>0.18</v>
@@ -19445,24 +19469,30 @@
       </c>
       <c r="T123" s="52" t="n">
         <f aca="false">IF(S123="IGST",ROUND(Q123*R123,2),0)</f>
+        <v>8052.32</v>
       </c>
       <c r="U123" s="52" t="n">
         <f aca="false">IF(S123="CGST+SGST",ROUND(Q123*R123/2,2),0)</f>
+        <v>0.0</v>
       </c>
       <c r="V123" s="52" t="n">
         <f aca="false">U123</f>
+        <v>0.0</v>
       </c>
       <c r="W123" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="X123" s="52" t="n">
         <f aca="false">Q123+T123+U123+V123+W123</f>
+        <v>52787.45</v>
       </c>
       <c r="Y123" s="52" t="n">
         <f aca="false">ROUND(Q123*AT123,0)</f>
+        <v>895.0</v>
       </c>
       <c r="Z123" s="52" t="n">
         <f aca="false">X123-Y123</f>
+        <v>51892.45</v>
       </c>
       <c r="AA123" s="47"/>
       <c r="AB123" s="47"/>
@@ -19479,7 +19509,7 @@
       </c>
       <c r="AF123" s="47" t="inlineStr">
         <is>
-          <t>Delhi (07)</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="AG123" s="47"/>
@@ -19495,12 +19525,12 @@
       <c r="AQ123" s="47"/>
       <c r="AR123" s="47" t="inlineStr">
         <is>
-          <t>No RCM – forward charge; goods/services, IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
+          <t>No RCM - forward charge; IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
         </is>
       </c>
       <c r="AS123" s="47" t="inlineStr">
         <is>
-          <t>Sec 393(1) – contract/service (old 194C), 2% (company). Confirm with CA.</t>
+          <t>194I</t>
         </is>
       </c>
       <c r="AT123" s="54" t="n">
@@ -19509,7 +19539,7 @@
     </row>
     <row r="124" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="47" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B124" s="47" t="inlineStr">
         <is>
@@ -19518,7 +19548,7 @@
       </c>
       <c r="C124" s="47" t="inlineStr">
         <is>
-          <t>IND/450459</t>
+          <t>IND-450459</t>
         </is>
       </c>
       <c r="D124" s="48" t="n">
@@ -19526,9 +19556,11 @@
       </c>
       <c r="E124" s="49" t="n">
         <f aca="false">YEAR(D124)</f>
+        <v>2026</v>
       </c>
       <c r="F124" s="50" t="str">
         <f aca="false">TEXT(D124,"mmm")</f>
+        <v>Oct</v>
       </c>
       <c r="G124" s="47" t="inlineStr">
         <is>
@@ -19543,10 +19575,14 @@
       <c r="I124" s="47"/>
       <c r="J124" s="47" t="inlineStr">
         <is>
-          <t>Expense / Services - Mahindra &amp; Mahindra Financial Services Limited</t>
+          <t>FMS Rental - Kia Sonet 1.0 T-GDI HTX DCT Petrol _ HR26FR5339 110949-1 ARUN KUMAR PANIGRAHI NBE00141 1 0</t>
         </is>
       </c>
-      <c r="K124" s="55"/>
+      <c r="K124" s="55" t="inlineStr">
+        <is>
+          <t>996749</t>
+        </is>
+      </c>
       <c r="L124" s="47"/>
       <c r="M124" s="47" t="n">
         <v>1.0</v>
@@ -19557,13 +19593,14 @@
         </is>
       </c>
       <c r="O124" s="51" t="n">
-        <v>121349.22</v>
+        <v>2522.14</v>
       </c>
       <c r="P124" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="Q124" s="52" t="n">
         <f aca="false">M124*O124-P124</f>
+        <v>2522.14</v>
       </c>
       <c r="R124" s="53" t="n">
         <v>0.18</v>
@@ -19575,24 +19612,30 @@
       </c>
       <c r="T124" s="52" t="n">
         <f aca="false">IF(S124="IGST",ROUND(Q124*R124,2),0)</f>
+        <v>453.99</v>
       </c>
       <c r="U124" s="52" t="n">
         <f aca="false">IF(S124="CGST+SGST",ROUND(Q124*R124/2,2),0)</f>
+        <v>0.0</v>
       </c>
       <c r="V124" s="52" t="n">
         <f aca="false">U124</f>
+        <v>0.0</v>
       </c>
       <c r="W124" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="X124" s="52" t="n">
         <f aca="false">Q124+T124+U124+V124+W124</f>
+        <v>2976.13</v>
       </c>
       <c r="Y124" s="52" t="n">
         <f aca="false">ROUND(Q124*AT124,0)</f>
+        <v>50.0</v>
       </c>
       <c r="Z124" s="52" t="n">
         <f aca="false">X124-Y124</f>
+        <v>2926.13</v>
       </c>
       <c r="AA124" s="47"/>
       <c r="AB124" s="47"/>
@@ -19625,12 +19668,12 @@
       <c r="AQ124" s="47"/>
       <c r="AR124" s="47" t="inlineStr">
         <is>
-          <t>No RCM – forward charge; goods/services, IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
+          <t>No RCM - forward charge; IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
         </is>
       </c>
       <c r="AS124" s="47" t="inlineStr">
         <is>
-          <t>Sec 393(1) – contract/service (old 194C), 2% (company). Confirm with CA.</t>
+          <t>194I</t>
         </is>
       </c>
       <c r="AT124" s="54" t="n">
@@ -19639,44 +19682,50 @@
     </row>
     <row r="125" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="47" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B125" s="47" t="inlineStr">
         <is>
-          <t>XTO10X Technologies Private Limited\2026-27-224 01.10.26.pdf</t>
+          <t>Mahindra &amp; Mahindra Financial Services Limited\IND-450459 01.10.26.pdf</t>
         </is>
       </c>
       <c r="C125" s="47" t="inlineStr">
         <is>
-          <t>2026-27/224</t>
+          <t>IND-450459</t>
         </is>
       </c>
       <c r="D125" s="48" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E125" s="49" t="n">
-        <f aca="false">YEAR(D122)</f>
+        <f aca="false">YEAR(D125)</f>
+        <v>2026</v>
       </c>
       <c r="F125" s="50" t="str">
-        <f aca="false">TEXT(D122,"mmm")</f>
+        <f aca="false">TEXT(D125,"mmm")</f>
+        <v>Oct</v>
       </c>
       <c r="G125" s="47" t="inlineStr">
         <is>
-          <t>XTO10X Technologies Private Limited</t>
+          <t>Mahindra &amp; Mahindra Financial Services Limited</t>
         </is>
       </c>
       <c r="H125" s="47" t="inlineStr">
         <is>
-          <t>29AAACX2697R1Z9</t>
+          <t>27AAACM2931R3Z1</t>
         </is>
       </c>
       <c r="I125" s="47"/>
       <c r="J125" s="47" t="inlineStr">
         <is>
-          <t>Expense / Services - XTO10X Technologies Private Limited</t>
+          <t>Lease Rental - Audi Q3 Sportback 40 TFSI Bold Edition Petrol Automatic DL3CDD0876 110949-2 Shashi Kapoor NBE0053</t>
         </is>
       </c>
-      <c r="K125" s="55"/>
+      <c r="K125" s="55" t="inlineStr">
+        <is>
+          <t>997319</t>
+        </is>
+      </c>
       <c r="L125" s="47"/>
       <c r="M125" s="47" t="n">
         <v>1.0</v>
@@ -19687,16 +19736,17 @@
         </is>
       </c>
       <c r="O125" s="51" t="n">
-        <v>847457.63</v>
+        <v>85656.05</v>
       </c>
       <c r="P125" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="Q125" s="52" t="n">
-        <f aca="false">M122*O122-P122</f>
+        <f aca="false">M125*O125-P125</f>
+        <v>85656.05</v>
       </c>
       <c r="R125" s="53" t="n">
-        <v>0.18</v>
+        <v>0.4</v>
       </c>
       <c r="S125" s="47" t="inlineStr">
         <is>
@@ -19704,42 +19754,48 @@
         </is>
       </c>
       <c r="T125" s="52" t="n">
-        <f aca="false">IF(S122="IGST",ROUND(Q122*R122,2),0)</f>
+        <f aca="false">IF(S125="IGST",ROUND(Q125*R125,2),0)</f>
+        <v>34262.42</v>
       </c>
       <c r="U125" s="52" t="n">
-        <f aca="false">IF(S122="CGST+SGST",ROUND(Q122*R122/2,2),0)</f>
+        <f aca="false">IF(S125="CGST+SGST",ROUND(Q125*R125/2,2),0)</f>
+        <v>0.0</v>
       </c>
       <c r="V125" s="52" t="n">
-        <f aca="false">U122</f>
+        <f aca="false">U125</f>
+        <v>0.0</v>
       </c>
       <c r="W125" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="X125" s="52" t="n">
-        <f aca="false">Q122+T122+U122+V122+W122</f>
+        <f aca="false">Q125+T125+U125+V125+W125</f>
+        <v>119918.47</v>
       </c>
       <c r="Y125" s="52" t="n">
-        <f aca="false">ROUND(Q122*AT122,0)</f>
+        <f aca="false">ROUND(Q125*AT125,0)</f>
+        <v>1713.0</v>
       </c>
       <c r="Z125" s="52" t="n">
-        <f aca="false">X122-Y122</f>
+        <f aca="false">X125-Y125</f>
+        <v>118205.47</v>
       </c>
       <c r="AA125" s="47"/>
       <c r="AB125" s="47"/>
       <c r="AC125" s="47"/>
       <c r="AD125" s="47" t="inlineStr">
         <is>
-          <t>Karnataka (29)</t>
+          <t>Maharashtra (27)</t>
         </is>
       </c>
       <c r="AE125" s="47" t="inlineStr">
         <is>
-          <t>07AAFCN6567R2ZI</t>
+          <t>07AAFCN6567R1ZJ</t>
         </is>
       </c>
       <c r="AF125" s="47" t="inlineStr">
         <is>
-          <t>Delhi (07)</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="AG125" s="47"/>
@@ -19755,12 +19811,12 @@
       <c r="AQ125" s="47"/>
       <c r="AR125" s="47" t="inlineStr">
         <is>
-          <t>No RCM – forward charge; goods/services, IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
+          <t>No RCM - forward charge; IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
         </is>
       </c>
       <c r="AS125" s="47" t="inlineStr">
         <is>
-          <t>Sec 393(1) – contract/service (old 194C), 2% (company). Confirm with CA.</t>
+          <t>194I</t>
         </is>
       </c>
       <c r="AT125" s="54" t="n">
@@ -19769,26 +19825,28 @@
     </row>
     <row r="126" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="47" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B126" s="47" t="inlineStr">
         <is>
-          <t>Mahindra &amp; Mahindra Financial Services Limited\NICOBAR DESIGN PRIVATE LIMITED_Oct 26_Reimbursement_231742 02.10.26.pdf</t>
+          <t>Mahindra &amp; Mahindra Financial Services Limited\IND-450459 01.10.26.pdf</t>
         </is>
       </c>
       <c r="C126" s="47" t="inlineStr">
         <is>
-          <t>NICOBAR DESIGN PRIVATE LIMITED_Oct 26_Reimbursement_231742</t>
+          <t>IND-450459</t>
         </is>
       </c>
       <c r="D126" s="48" t="n">
         <v>46297</v>
       </c>
       <c r="E126" s="49" t="n">
-        <f aca="false">YEAR(D123)</f>
+        <f aca="false">YEAR(D126)</f>
+        <v>2026</v>
       </c>
       <c r="F126" s="50" t="str">
-        <f aca="false">TEXT(D123,"mmm")</f>
+        <f aca="false">TEXT(D126,"mmm")</f>
+        <v>Oct</v>
       </c>
       <c r="G126" s="47" t="inlineStr">
         <is>
@@ -19803,10 +19861,14 @@
       <c r="I126" s="47"/>
       <c r="J126" s="47" t="inlineStr">
         <is>
-          <t>Expense / Services - Mahindra &amp; Mahindra Financial Services Limited</t>
+          <t>FMS Rental - Audi Q3 Sportback 40 TFSI Bold Edition Petrol Automatic DL3CDD0876 110949-2 Shashi Kapoor NBE0053 1 0</t>
         </is>
       </c>
-      <c r="K126" s="55"/>
+      <c r="K126" s="55" t="inlineStr">
+        <is>
+          <t>996749</t>
+        </is>
+      </c>
       <c r="L126" s="47"/>
       <c r="M126" s="47" t="n">
         <v>1.0</v>
@@ -19817,13 +19879,14 @@
         </is>
       </c>
       <c r="O126" s="51" t="n">
-        <v>20506.19</v>
+        <v>10278.76</v>
       </c>
       <c r="P126" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="Q126" s="52" t="n">
-        <f aca="false">M123*O123-P123</f>
+        <f aca="false">M126*O126-P126</f>
+        <v>10278.76</v>
       </c>
       <c r="R126" s="53" t="n">
         <v>0.18</v>
@@ -19834,25 +19897,31 @@
         </is>
       </c>
       <c r="T126" s="52" t="n">
-        <f aca="false">IF(S123="IGST",ROUND(Q123*R123,2),0)</f>
+        <f aca="false">IF(S126="IGST",ROUND(Q126*R126,2),0)</f>
+        <v>1850.18</v>
       </c>
       <c r="U126" s="52" t="n">
-        <f aca="false">IF(S123="CGST+SGST",ROUND(Q123*R123/2,2),0)</f>
+        <f aca="false">IF(S126="CGST+SGST",ROUND(Q126*R126/2,2),0)</f>
+        <v>0.0</v>
       </c>
       <c r="V126" s="52" t="n">
-        <f aca="false">U123</f>
+        <f aca="false">U126</f>
+        <v>0.0</v>
       </c>
       <c r="W126" s="51" t="n">
-        <v>0.0</v>
+        <v>0.01</v>
       </c>
       <c r="X126" s="52" t="n">
-        <f aca="false">Q123+T123+U123+V123+W123</f>
+        <f aca="false">Q126+T126+U126+V126+W126</f>
+        <v>12128.95</v>
       </c>
       <c r="Y126" s="52" t="n">
-        <f aca="false">ROUND(Q123*AT123,0)</f>
+        <f aca="false">ROUND(Q126*AT126,0)</f>
+        <v>206.0</v>
       </c>
       <c r="Z126" s="52" t="n">
-        <f aca="false">X123-Y123</f>
+        <f aca="false">X126-Y126</f>
+        <v>11922.95</v>
       </c>
       <c r="AA126" s="47"/>
       <c r="AB126" s="47"/>
@@ -19869,7 +19938,7 @@
       </c>
       <c r="AF126" s="47" t="inlineStr">
         <is>
-          <t>Delhi (07)</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="AG126" s="47"/>
@@ -19885,12 +19954,12 @@
       <c r="AQ126" s="47"/>
       <c r="AR126" s="47" t="inlineStr">
         <is>
-          <t>No RCM – forward charge; goods/services, IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
+          <t>No RCM - forward charge; IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
         </is>
       </c>
       <c r="AS126" s="47" t="inlineStr">
         <is>
-          <t>Sec 393(1) – contract/service (old 194C), 2% (company). Confirm with CA.</t>
+          <t>194I</t>
         </is>
       </c>
       <c r="AT126" s="54" t="n">
@@ -19899,26 +19968,28 @@
     </row>
     <row r="127" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="47" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B127" s="47" t="inlineStr">
         <is>
-          <t>Mahindra &amp; Mahindra Financial Services Limited\NICOBAR DESIGN PRIVATE LIMITED_Oct 26_FMS Rental_Lease Rental_IND-450459 02.10.26.pdf</t>
+          <t>Mahindra &amp; Mahindra Financial Services Limited\231742 01.10.26.pdf</t>
         </is>
       </c>
       <c r="C127" s="47" t="inlineStr">
         <is>
-          <t>NICOBAR DESIGN PRIVATE LIMITED_Oct 26_FMS Rental_Lease Rental_IND/450459</t>
+          <t>231742</t>
         </is>
       </c>
       <c r="D127" s="48" t="n">
         <v>46297</v>
       </c>
       <c r="E127" s="49" t="n">
-        <f aca="false">YEAR(D124)</f>
+        <f aca="false">YEAR(D127)</f>
+        <v>2026</v>
       </c>
       <c r="F127" s="50" t="str">
-        <f aca="false">TEXT(D124,"mmm")</f>
+        <f aca="false">TEXT(D127,"mmm")</f>
+        <v>Oct</v>
       </c>
       <c r="G127" s="47" t="inlineStr">
         <is>
@@ -19933,7 +20004,7 @@
       <c r="I127" s="47"/>
       <c r="J127" s="47" t="inlineStr">
         <is>
-          <t>Expense / Services - Mahindra &amp; Mahindra Financial Services Limited</t>
+          <t>Mahindra &amp; Mahindra Financial Services Limited - invoice 231742</t>
         </is>
       </c>
       <c r="K127" s="55"/>
@@ -19947,16 +20018,17 @@
         </is>
       </c>
       <c r="O127" s="51" t="n">
-        <v>121349.22</v>
+        <v>24197.3</v>
       </c>
       <c r="P127" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="Q127" s="52" t="n">
-        <f aca="false">M124*O124-P124</f>
+        <f aca="false">M127*O127-P127</f>
+        <v>24197.3</v>
       </c>
       <c r="R127" s="53" t="n">
-        <v>0.18</v>
+        <v>0.0</v>
       </c>
       <c r="S127" s="47" t="inlineStr">
         <is>
@@ -19964,25 +20036,31 @@
         </is>
       </c>
       <c r="T127" s="52" t="n">
-        <f aca="false">IF(S124="IGST",ROUND(Q124*R124,2),0)</f>
+        <f aca="false">IF(S127="IGST",ROUND(Q127*R127,2),0)</f>
+        <v>0.0</v>
       </c>
       <c r="U127" s="52" t="n">
-        <f aca="false">IF(S124="CGST+SGST",ROUND(Q124*R124/2,2),0)</f>
+        <f aca="false">IF(S127="CGST+SGST",ROUND(Q127*R127/2,2),0)</f>
+        <v>0.0</v>
       </c>
       <c r="V127" s="52" t="n">
-        <f aca="false">U124</f>
+        <f aca="false">U127</f>
+        <v>0.0</v>
       </c>
       <c r="W127" s="51" t="n">
-        <v>0.0</v>
+        <v>0.7</v>
       </c>
       <c r="X127" s="52" t="n">
-        <f aca="false">Q124+T124+U124+V124+W124</f>
+        <f aca="false">Q127+T127+U127+V127+W127</f>
+        <v>24198.0</v>
       </c>
       <c r="Y127" s="52" t="n">
-        <f aca="false">ROUND(Q124*AT124,0)</f>
+        <f aca="false">ROUND(Q127*AT127,0)</f>
+        <v>484.0</v>
       </c>
       <c r="Z127" s="52" t="n">
-        <f aca="false">X124-Y124</f>
+        <f aca="false">X127-Y127</f>
+        <v>23714.0</v>
       </c>
       <c r="AA127" s="47"/>
       <c r="AB127" s="47"/>
@@ -19999,7 +20077,7 @@
       </c>
       <c r="AF127" s="47" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Delhi (07)</t>
         </is>
       </c>
       <c r="AG127" s="47"/>
@@ -20015,12 +20093,12 @@
       <c r="AQ127" s="47"/>
       <c r="AR127" s="47" t="inlineStr">
         <is>
-          <t>No RCM – forward charge; goods/services, IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
+          <t>No RCM - forward charge; IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
         </is>
       </c>
       <c r="AS127" s="47" t="inlineStr">
         <is>
-          <t>Sec 393(1) – contract/service (old 194C), 2% (company). Confirm with CA.</t>
+          <t>194I</t>
         </is>
       </c>
       <c r="AT127" s="54" t="n">
@@ -20029,37 +20107,43 @@
     </row>
     <row r="128" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="47" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B128" s="47" t="inlineStr">
         <is>
-          <t>General Expenses\WhatsApp Image 2026-10-01 at 2.50.38 PM 04.10.26.pdf</t>
+          <t>Niva's Designs\ND-26-27-043 29.07.26.pdf</t>
         </is>
       </c>
       <c r="C128" s="47" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026/10/01 at 2.50.38 PM</t>
+          <t>ND/26-27/043</t>
         </is>
       </c>
       <c r="D128" s="48" t="n">
-        <v>46299</v>
+        <v>46232</v>
       </c>
       <c r="E128" s="49" t="n">
-        <f aca="false">YEAR(D125)</f>
+        <f aca="false">YEAR(D128)</f>
+        <v>2026</v>
       </c>
       <c r="F128" s="50" t="str">
-        <f aca="false">TEXT(D125,"mmm")</f>
+        <f aca="false">TEXT(D128,"mmm")</f>
+        <v>Jul</v>
       </c>
       <c r="G128" s="47" t="inlineStr">
         <is>
-          <t>General Expenses</t>
+          <t>Niva's Designs</t>
         </is>
       </c>
-      <c r="H128" s="47"/>
+      <c r="H128" s="47" t="inlineStr">
+        <is>
+          <t>06BCAPS9611Q1Z0</t>
+        </is>
+      </c>
       <c r="I128" s="47"/>
       <c r="J128" s="47" t="inlineStr">
         <is>
-          <t>Expense / Services - General Expenses</t>
+          <t>Niva's Designs - invoice ND/26-27/043</t>
         </is>
       </c>
       <c r="K128" s="55"/>
@@ -20073,55 +20157,66 @@
         </is>
       </c>
       <c r="O128" s="51" t="n">
-        <v>0.0</v>
+        <v>33846.2</v>
       </c>
       <c r="P128" s="51" t="n">
         <v>0.0</v>
       </c>
       <c r="Q128" s="52" t="n">
-        <f aca="false">M125*O125-P125</f>
+        <f aca="false">M128*O128-P128</f>
+        <v>33846.2</v>
       </c>
       <c r="R128" s="53" t="n">
-        <v>0.0</v>
+        <v>0.05</v>
       </c>
       <c r="S128" s="47" t="inlineStr">
         <is>
-          <t>No GST (unregistered)</t>
+          <t>IGST</t>
         </is>
       </c>
       <c r="T128" s="52" t="n">
-        <f aca="false">IF(S125="IGST",ROUND(Q125*R125,2),0)</f>
+        <f aca="false">IF(S128="IGST",ROUND(Q128*R128,2),0)</f>
+        <v>1692.31</v>
       </c>
       <c r="U128" s="52" t="n">
-        <f aca="false">IF(S125="CGST+SGST",ROUND(Q125*R125/2,2),0)</f>
+        <f aca="false">IF(S128="CGST+SGST",ROUND(Q128*R128/2,2),0)</f>
+        <v>0.0</v>
       </c>
       <c r="V128" s="52" t="n">
-        <f aca="false">U125</f>
+        <f aca="false">U128</f>
+        <v>0.0</v>
       </c>
       <c r="W128" s="51" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="X128" s="52" t="n">
+        <f aca="false">Q128+T128+U128+V128+W128</f>
+        <v>35539.0</v>
+      </c>
+      <c r="Y128" s="52" t="n">
+        <f aca="false">ROUND(Q128*AT128,0)</f>
         <v>0.0</v>
       </c>
-      <c r="X128" s="52" t="n">
-        <f aca="false">Q125+T125+U125+V125+W125</f>
-      </c>
-      <c r="Y128" s="52" t="n">
-        <f aca="false">ROUND(Q125*AT125,0)</f>
-      </c>
       <c r="Z128" s="52" t="n">
-        <f aca="false">X125-Y125</f>
+        <f aca="false">X128-Y128</f>
+        <v>35539.0</v>
       </c>
       <c r="AA128" s="47"/>
       <c r="AB128" s="47"/>
       <c r="AC128" s="47"/>
-      <c r="AD128" s="47"/>
+      <c r="AD128" s="47" t="inlineStr">
+        <is>
+          <t>Haryana (06)</t>
+        </is>
+      </c>
       <c r="AE128" s="47" t="inlineStr">
         <is>
-          <t>06AAFCN6567R1ZL</t>
+          <t>07AAFCN6567R1ZJ</t>
         </is>
       </c>
       <c r="AF128" s="47" t="inlineStr">
         <is>
-          <t>Haryana (06)</t>
+          <t>Delhi (07)</t>
         </is>
       </c>
       <c r="AG128" s="47"/>
@@ -20137,1016 +20232,114 @@
       <c r="AQ128" s="47"/>
       <c r="AR128" s="47" t="inlineStr">
         <is>
-          <t>No RCM – forward charge; CGST + SGST charged by supplier. ITC eligible (check GSTR-2B).</t>
-        </is>
-      </c>
-      <c r="AS128" s="47" t="inlineStr">
-        <is>
-          <t>Sec 393(1) – purchase of goods (old 194Q), code 1031. Apply only if FY purchases from this supplier &gt; ₹50 L (on excess).</t>
-        </is>
-      </c>
-      <c r="AT128" s="54" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A129" s="47" t="n">
-        <v>122</v>
-      </c>
-      <c r="B129" s="47" t="inlineStr">
-        <is>
-          <t>Curefoods India Limited\BIN-2026- 02.10.26.pdf</t>
-        </is>
-      </c>
-      <c r="C129" s="47" t="inlineStr">
-        <is>
-          <t>BIN/2026-</t>
-        </is>
-      </c>
-      <c r="D129" s="48" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E129" s="49" t="n">
-        <f aca="false">YEAR(D126)</f>
-      </c>
-      <c r="F129" s="50" t="str">
-        <f aca="false">TEXT(D126,"mmm")</f>
-      </c>
-      <c r="G129" s="47" t="inlineStr">
-        <is>
-          <t>Curefoods India Limited</t>
-        </is>
-      </c>
-      <c r="H129" s="47" t="inlineStr">
-        <is>
-          <t>29AAJCC0315J1ZQ</t>
-        </is>
-      </c>
-      <c r="I129" s="47"/>
-      <c r="J129" s="47" t="inlineStr">
-        <is>
-          <t>Expense / Services - Curefoods India Limited</t>
-        </is>
-      </c>
-      <c r="K129" s="55"/>
-      <c r="L129" s="47"/>
-      <c r="M129" s="47" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="N129" s="47" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="O129" s="51" t="n">
-        <v>17137.71</v>
-      </c>
-      <c r="P129" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Q129" s="52" t="n">
-        <f aca="false">M126*O126-P126</f>
-      </c>
-      <c r="R129" s="53" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="S129" s="47" t="inlineStr">
-        <is>
-          <t>IGST</t>
-        </is>
-      </c>
-      <c r="T129" s="52" t="n">
-        <f aca="false">IF(S126="IGST",ROUND(Q126*R126,2),0)</f>
-      </c>
-      <c r="U129" s="52" t="n">
-        <f aca="false">IF(S126="CGST+SGST",ROUND(Q126*R126/2,2),0)</f>
-      </c>
-      <c r="V129" s="52" t="n">
-        <f aca="false">U126</f>
-      </c>
-      <c r="W129" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="X129" s="52" t="n">
-        <f aca="false">Q126+T126+U126+V126+W126</f>
-      </c>
-      <c r="Y129" s="52" t="n">
-        <f aca="false">ROUND(Q126*AT126,0)</f>
-      </c>
-      <c r="Z129" s="52" t="n">
-        <f aca="false">X126-Y126</f>
-      </c>
-      <c r="AA129" s="47"/>
-      <c r="AB129" s="47"/>
-      <c r="AC129" s="47"/>
-      <c r="AD129" s="47" t="inlineStr">
-        <is>
-          <t>Karnataka (29)</t>
-        </is>
-      </c>
-      <c r="AE129" s="47" t="inlineStr">
-        <is>
-          <t>06AAFCN6567R1ZL</t>
-        </is>
-      </c>
-      <c r="AF129" s="47" t="inlineStr">
-        <is>
-          <t>Haryana (06)</t>
-        </is>
-      </c>
-      <c r="AG129" s="47"/>
-      <c r="AH129" s="48"/>
-      <c r="AI129" s="47"/>
-      <c r="AJ129" s="47"/>
-      <c r="AK129" s="47"/>
-      <c r="AL129" s="47"/>
-      <c r="AM129" s="47"/>
-      <c r="AN129" s="47"/>
-      <c r="AO129" s="47"/>
-      <c r="AP129" s="47"/>
-      <c r="AQ129" s="47"/>
-      <c r="AR129" s="47" t="inlineStr">
-        <is>
-          <t>No RCM – forward charge; goods/services, IGST charged by supplier. ITC eligible (check GSTR-2B).</t>
-        </is>
-      </c>
-      <c r="AS129" s="47" t="inlineStr">
-        <is>
-          <t>Sec 393(1) – purchase of goods (old 194Q), code 1031. Apply only if FY purchases from this supplier &gt; ₹50 L (on excess).</t>
-        </is>
-      </c>
-      <c r="AT129" s="54" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A130" s="47" t="n">
-        <v>123</v>
-      </c>
-      <c r="B130" s="47" t="inlineStr">
-        <is>
-          <t>Niva's Designs\CN_Nicobar_Delhi_29-08-26 04.10.26.pdf</t>
-        </is>
-      </c>
-      <c r="C130" s="47" t="inlineStr">
-        <is>
-          <t>CN_Nicobar_Delhi_29/08/26</t>
-        </is>
-      </c>
-      <c r="D130" s="48" t="n">
-        <v>46299</v>
-      </c>
-      <c r="E130" s="49" t="n">
-        <f aca="false">YEAR(D127)</f>
-      </c>
-      <c r="F130" s="50" t="str">
-        <f aca="false">TEXT(D127,"mmm")</f>
-      </c>
-      <c r="G130" s="47" t="inlineStr">
-        <is>
-          <t>Niva's Designs</t>
-        </is>
-      </c>
-      <c r="H130" s="47" t="inlineStr">
-        <is>
-          <t>06BCAPS9611Q1Z0</t>
-        </is>
-      </c>
-      <c r="I130" s="47"/>
-      <c r="J130" s="47" t="inlineStr">
-        <is>
-          <t>Expense / Services - Niva's Designs</t>
-        </is>
-      </c>
-      <c r="K130" s="55"/>
-      <c r="L130" s="47"/>
-      <c r="M130" s="47" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="N130" s="47" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="O130" s="51" t="n">
-        <v>30117.8</v>
-      </c>
-      <c r="P130" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Q130" s="52" t="n">
-        <f aca="false">M127*O127-P127</f>
-      </c>
-      <c r="R130" s="53" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="S130" s="47" t="inlineStr">
-        <is>
-          <t>IGST</t>
-        </is>
-      </c>
-      <c r="T130" s="52" t="n">
-        <f aca="false">IF(S127="IGST",ROUND(Q127*R127,2),0)</f>
-      </c>
-      <c r="U130" s="52" t="n">
-        <f aca="false">IF(S127="CGST+SGST",ROUND(Q127*R127/2,2),0)</f>
-      </c>
-      <c r="V130" s="52" t="n">
-        <f aca="false">U127</f>
-      </c>
-      <c r="W130" s="51" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="X130" s="52" t="n">
-        <f aca="false">Q127+T127+U127+V127+W127</f>
-      </c>
-      <c r="Y130" s="52" t="n">
-        <f aca="false">ROUND(Q127*AT127,0)</f>
-      </c>
-      <c r="Z130" s="52" t="n">
-        <f aca="false">X127-Y127</f>
-      </c>
-      <c r="AA130" s="47"/>
-      <c r="AB130" s="47"/>
-      <c r="AC130" s="47"/>
-      <c r="AD130" s="47" t="inlineStr">
-        <is>
-          <t>Haryana (06)</t>
-        </is>
-      </c>
-      <c r="AE130" s="47" t="inlineStr">
-        <is>
-          <t>07AAFCN6567R1ZJ</t>
-        </is>
-      </c>
-      <c r="AF130" s="47" t="inlineStr">
-        <is>
-          <t>Delhi (07)</t>
-        </is>
-      </c>
-      <c r="AG130" s="47" t="inlineStr">
-        <is>
-          <t>Dispatch</t>
-        </is>
-      </c>
-      <c r="AH130" s="48"/>
-      <c r="AI130" s="47"/>
-      <c r="AJ130" s="47"/>
-      <c r="AK130" s="47"/>
-      <c r="AL130" s="47"/>
-      <c r="AM130" s="47"/>
-      <c r="AN130" s="47"/>
-      <c r="AO130" s="47"/>
-      <c r="AP130" s="47"/>
-      <c r="AQ130" s="47"/>
-      <c r="AR130" s="47" t="inlineStr">
-        <is>
           <t>No RCM – forward charge; goods, CGST 2.5% + SGST 2.5%. ITC eligible (check GSTR-2B). Re-issued to Haryana GSTIN – invoice says actual invoice date 29-07-2026. Original ND/26-27/043 (Delhi, IGST) cancelled by credit note ND/26-27/CN3 – not entered. PO no./date taken from email thread. Nicobar asked for LR copy for ₹650 freight. Terms 45 days.</t>
         </is>
       </c>
-      <c r="AS130" s="47" t="inlineStr">
+      <c r="AS128" s="47" t="inlineStr">
         <is>
           <t>Sec 393(1) – purchase of goods (old 194Q). Apply only if FY purchases from this supplier &gt; ₹50 L – nil assumed.</t>
         </is>
       </c>
-      <c r="AT130" s="54" t="n">
-        <v>0</v>
+      <c r="AT128" s="54" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A130" s="44"/>
+      <c r="B130" s="44"/>
+      <c r="C130" s="44"/>
+      <c r="D130" s="44"/>
+      <c r="E130" s="44"/>
+      <c r="F130" s="44"/>
+      <c r="G130" s="44"/>
+      <c r="H130" s="44"/>
+      <c r="I130" s="44"/>
+      <c r="J130" s="44"/>
+      <c r="K130" s="44"/>
+      <c r="L130" s="44"/>
+      <c r="M130" s="44"/>
+      <c r="N130" s="44"/>
+      <c r="O130" s="44"/>
+      <c r="P130" s="56" t="s">
+        <v>667</v>
+      </c>
+      <c r="Q130" s="57" t="n">
+        <f aca="false">SUM(Q5:Q129)</f>
+        <v>9351896.08564</v>
+      </c>
+      <c r="R130" s="44"/>
+      <c r="S130" s="44"/>
+      <c r="T130" s="57" t="n">
+        <f aca="false">SUM(T5:T129)</f>
+        <v>664878.33</v>
+      </c>
+      <c r="U130" s="57" t="n">
+        <f aca="false">SUM(U5:U129)</f>
+        <v>338408.52</v>
+      </c>
+      <c r="V130" s="57" t="n">
+        <f aca="false">SUM(V5:V129)</f>
+        <v>338408.52</v>
+      </c>
+      <c r="W130" s="57" t="n">
+        <f aca="false">SUM(W5:W129)</f>
+        <v>2.18</v>
+      </c>
+      <c r="X130" s="57" t="n">
+        <f aca="false">SUM(X5:X129)</f>
+        <v>10693593.63564</v>
+      </c>
+      <c r="Y130" s="57" t="n">
+        <f aca="false">SUM(Y5:Y129)</f>
+        <v>313579.0</v>
+      </c>
+      <c r="Z130" s="57" t="n">
+        <f aca="false">SUM(Z5:Z129)</f>
+        <v>10380014.63564</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A131" s="47" t="n">
-        <v>124</v>
-      </c>
-      <c r="B131" s="47" t="inlineStr">
-        <is>
-          <t>Niva's Designs\ND-26-27-043 04.10.26.pdf</t>
-        </is>
-      </c>
-      <c r="C131" s="47" t="inlineStr">
-        <is>
-          <t>ND/26-27/043</t>
-        </is>
-      </c>
-      <c r="D131" s="48" t="n">
-        <v>46299</v>
-      </c>
-      <c r="E131" s="49" t="n">
-        <f aca="false">YEAR(D128)</f>
-      </c>
-      <c r="F131" s="50" t="str">
-        <f aca="false">TEXT(D128,"mmm")</f>
-      </c>
-      <c r="G131" s="47" t="inlineStr">
-        <is>
-          <t>Niva's Designs</t>
-        </is>
-      </c>
-      <c r="H131" s="47" t="inlineStr">
-        <is>
-          <t>06BCAPS9611Q1Z0</t>
-        </is>
-      </c>
-      <c r="I131" s="47"/>
-      <c r="J131" s="47" t="inlineStr">
-        <is>
-          <t>Expense / Services - Niva's Designs</t>
-        </is>
-      </c>
-      <c r="K131" s="55"/>
-      <c r="L131" s="47"/>
-      <c r="M131" s="47" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="N131" s="47" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="O131" s="51" t="n">
-        <v>30117.8</v>
-      </c>
-      <c r="P131" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Q131" s="52" t="n">
-        <f aca="false">M128*O128-P128</f>
-      </c>
-      <c r="R131" s="53" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="S131" s="47" t="inlineStr">
-        <is>
-          <t>IGST</t>
-        </is>
-      </c>
-      <c r="T131" s="52" t="n">
-        <f aca="false">IF(S128="IGST",ROUND(Q128*R128,2),0)</f>
-      </c>
-      <c r="U131" s="52" t="n">
-        <f aca="false">IF(S128="CGST+SGST",ROUND(Q128*R128/2,2),0)</f>
-      </c>
-      <c r="V131" s="52" t="n">
-        <f aca="false">U128</f>
-      </c>
-      <c r="W131" s="51" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="X131" s="52" t="n">
-        <f aca="false">Q128+T128+U128+V128+W128</f>
-      </c>
-      <c r="Y131" s="52" t="n">
-        <f aca="false">ROUND(Q128*AT128,0)</f>
-      </c>
-      <c r="Z131" s="52" t="n">
-        <f aca="false">X128-Y128</f>
-      </c>
-      <c r="AA131" s="47"/>
-      <c r="AB131" s="47"/>
-      <c r="AC131" s="47"/>
-      <c r="AD131" s="47" t="inlineStr">
-        <is>
-          <t>Haryana (06)</t>
-        </is>
-      </c>
-      <c r="AE131" s="47" t="inlineStr">
-        <is>
-          <t>07AAFCN6567R1ZJ</t>
-        </is>
-      </c>
-      <c r="AF131" s="47" t="inlineStr">
-        <is>
-          <t>Delhi (07)</t>
-        </is>
-      </c>
-      <c r="AG131" s="47" t="inlineStr">
-        <is>
-          <t>Dispatch</t>
-        </is>
-      </c>
-      <c r="AH131" s="48"/>
-      <c r="AI131" s="47" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="AJ131" s="47"/>
-      <c r="AK131" s="47"/>
-      <c r="AL131" s="47"/>
-      <c r="AM131" s="47"/>
-      <c r="AN131" s="47"/>
-      <c r="AO131" s="47"/>
-      <c r="AP131" s="47"/>
-      <c r="AQ131" s="47"/>
-      <c r="AR131" s="47" t="inlineStr">
-        <is>
-          <t>No RCM – forward charge; goods, CGST 2.5% + SGST 2.5%. ITC eligible (check GSTR-2B). Re-issued to Haryana GSTIN – invoice says actual invoice date 29-07-2026. Original ND/26-27/043 (Delhi, IGST) cancelled by credit note ND/26-27/CN3 – not entered. PO no./date taken from email thread. Nicobar asked for LR copy for ₹650 freight. Terms 45 days.</t>
-        </is>
-      </c>
-      <c r="AS131" s="47" t="inlineStr">
-        <is>
-          <t>Sec 393(1) – purchase of goods (old 194Q). Apply only if FY purchases from this supplier &gt; ₹50 L – nil assumed.</t>
-        </is>
-      </c>
-      <c r="AT131" s="54" t="n">
-        <v>0</v>
+      <c r="A131" s="45" t="s">
+        <v>668</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A132" s="47" t="n">
-        <v>125</v>
-      </c>
-      <c r="B132" s="47" t="inlineStr">
-        <is>
-          <t>IPinfo Inc\Invoice-3MNDSIX0-0003 (1) 04.10.26.pdf</t>
-        </is>
-      </c>
-      <c r="C132" s="47" t="inlineStr">
-        <is>
-          <t>Invoice/3MNDSIX0/0003 (1)</t>
-        </is>
-      </c>
-      <c r="D132" s="48" t="n">
-        <v>46299</v>
-      </c>
-      <c r="E132" s="49" t="n">
-        <f aca="false">YEAR(D129)</f>
-      </c>
-      <c r="F132" s="50" t="str">
-        <f aca="false">TEXT(D129,"mmm")</f>
-      </c>
-      <c r="G132" s="47" t="inlineStr">
-        <is>
-          <t>IPinfo Inc</t>
-        </is>
-      </c>
-      <c r="H132" s="47"/>
-      <c r="I132" s="47"/>
-      <c r="J132" s="47" t="inlineStr">
-        <is>
-          <t>Expense / Services - IPinfo Inc</t>
-        </is>
-      </c>
-      <c r="K132" s="55"/>
-      <c r="L132" s="47"/>
-      <c r="M132" s="47" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="N132" s="47" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="O132" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="P132" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Q132" s="52" t="n">
-        <f aca="false">M129*O129-P129</f>
-      </c>
-      <c r="R132" s="53" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="S132" s="47" t="inlineStr">
-        <is>
-          <t>No GST (unregistered)</t>
-        </is>
-      </c>
-      <c r="T132" s="52" t="n">
-        <f aca="false">IF(S129="IGST",ROUND(Q129*R129,2),0)</f>
-      </c>
-      <c r="U132" s="52" t="n">
-        <f aca="false">IF(S129="CGST+SGST",ROUND(Q129*R129/2,2),0)</f>
-      </c>
-      <c r="V132" s="52" t="n">
-        <f aca="false">U129</f>
-      </c>
-      <c r="W132" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="X132" s="52" t="n">
-        <f aca="false">Q129+T129+U129+V129+W129</f>
-      </c>
-      <c r="Y132" s="52" t="n">
-        <f aca="false">ROUND(Q129*AT129,0)</f>
-      </c>
-      <c r="Z132" s="52" t="n">
-        <f aca="false">X129-Y129</f>
-      </c>
-      <c r="AA132" s="47"/>
-      <c r="AB132" s="47"/>
-      <c r="AC132" s="47"/>
-      <c r="AD132" s="47"/>
-      <c r="AE132" s="47" t="inlineStr">
-        <is>
-          <t>06AAFCN6567R1ZL</t>
-        </is>
-      </c>
-      <c r="AF132" s="47" t="inlineStr">
-        <is>
-          <t>Haryana (06)</t>
-        </is>
-      </c>
-      <c r="AG132" s="47"/>
-      <c r="AH132" s="48"/>
-      <c r="AI132" s="47"/>
-      <c r="AJ132" s="47"/>
-      <c r="AK132" s="47"/>
-      <c r="AL132" s="47"/>
-      <c r="AM132" s="47"/>
-      <c r="AN132" s="47"/>
-      <c r="AO132" s="47"/>
-      <c r="AP132" s="47"/>
-      <c r="AQ132" s="47"/>
-      <c r="AR132" s="47" t="inlineStr">
-        <is>
-          <t>No RCM – forward charge; CGST + SGST charged by supplier. ITC eligible (check GSTR-2B).</t>
-        </is>
-      </c>
-      <c r="AS132" s="47" t="inlineStr">
-        <is>
-          <t>Sec 393(1) – purchase of goods (old 194Q), code 1031. Apply only if FY purchases from this supplier &gt; ₹50 L (on excess).</t>
-        </is>
-      </c>
-      <c r="AT132" s="54" t="n">
-        <v>0.001</v>
+      <c r="A132" s="45" t="s">
+        <v>669</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A133" s="47" t="n">
-        <v>126</v>
-      </c>
-      <c r="B133" s="47" t="inlineStr">
-        <is>
-          <t>General Expenses\WhatsApp Image 2026-09-29 at 3.31.47 PM 04.10.26.pdf</t>
-        </is>
-      </c>
-      <c r="C133" s="47" t="inlineStr">
-        <is>
-          <t>WhatsApp Image 2026/09/29 at 3.31.47 PM</t>
-        </is>
-      </c>
-      <c r="D133" s="48" t="n">
-        <v>46299</v>
-      </c>
-      <c r="E133" s="49" t="n">
-        <f aca="false">YEAR(D130)</f>
-      </c>
-      <c r="F133" s="50" t="str">
-        <f aca="false">TEXT(D130,"mmm")</f>
-      </c>
-      <c r="G133" s="47" t="inlineStr">
-        <is>
-          <t>General Expenses</t>
-        </is>
-      </c>
-      <c r="H133" s="47"/>
-      <c r="I133" s="47"/>
-      <c r="J133" s="47" t="inlineStr">
-        <is>
-          <t>Expense / Services - General Expenses</t>
-        </is>
-      </c>
-      <c r="K133" s="55"/>
-      <c r="L133" s="47"/>
-      <c r="M133" s="47" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="N133" s="47" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="O133" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="P133" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Q133" s="52" t="n">
-        <f aca="false">M130*O130-P130</f>
-      </c>
-      <c r="R133" s="53" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="S133" s="47" t="inlineStr">
-        <is>
-          <t>No GST (unregistered)</t>
-        </is>
-      </c>
-      <c r="T133" s="52" t="n">
-        <f aca="false">IF(S130="IGST",ROUND(Q130*R130,2),0)</f>
-      </c>
-      <c r="U133" s="52" t="n">
-        <f aca="false">IF(S130="CGST+SGST",ROUND(Q130*R130/2,2),0)</f>
-      </c>
-      <c r="V133" s="52" t="n">
-        <f aca="false">U130</f>
-      </c>
-      <c r="W133" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="X133" s="52" t="n">
-        <f aca="false">Q130+T130+U130+V130+W130</f>
-      </c>
-      <c r="Y133" s="52" t="n">
-        <f aca="false">ROUND(Q130*AT130,0)</f>
-      </c>
-      <c r="Z133" s="52" t="n">
-        <f aca="false">X130-Y130</f>
-      </c>
-      <c r="AA133" s="47"/>
-      <c r="AB133" s="47"/>
-      <c r="AC133" s="47"/>
-      <c r="AD133" s="47"/>
-      <c r="AE133" s="47" t="inlineStr">
-        <is>
-          <t>06AAFCN6567R1ZL</t>
-        </is>
-      </c>
-      <c r="AF133" s="47" t="inlineStr">
-        <is>
-          <t>Haryana (06)</t>
-        </is>
-      </c>
-      <c r="AG133" s="47"/>
-      <c r="AH133" s="48"/>
-      <c r="AI133" s="47"/>
-      <c r="AJ133" s="47"/>
-      <c r="AK133" s="47"/>
-      <c r="AL133" s="47"/>
-      <c r="AM133" s="47"/>
-      <c r="AN133" s="47"/>
-      <c r="AO133" s="47"/>
-      <c r="AP133" s="47"/>
-      <c r="AQ133" s="47"/>
-      <c r="AR133" s="47" t="inlineStr">
-        <is>
-          <t>No RCM – forward charge; CGST + SGST charged by supplier. ITC eligible (check GSTR-2B).</t>
-        </is>
-      </c>
-      <c r="AS133" s="47" t="inlineStr">
-        <is>
-          <t>Sec 393(1) – purchase of goods (old 194Q), code 1031. Apply only if FY purchases from this supplier &gt; ₹50 L (on excess).</t>
-        </is>
-      </c>
-      <c r="AT133" s="54" t="n">
-        <v>0.001</v>
+      <c r="A133" s="45" t="s">
+        <v>670</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A134" s="47" t="n">
-        <v>127</v>
-      </c>
-      <c r="B134" s="47" t="inlineStr">
-        <is>
-          <t>A &amp; S Creations\Invoice 065 - Nicobar - September 26 04.10.26.pdf</t>
-        </is>
-      </c>
-      <c r="C134" s="47" t="inlineStr">
-        <is>
-          <t>Invoice 065 / Nicobar / September 26</t>
-        </is>
-      </c>
-      <c r="D134" s="48" t="n">
-        <v>46299</v>
-      </c>
-      <c r="E134" s="49" t="n">
-        <f aca="false">YEAR(D131)</f>
-      </c>
-      <c r="F134" s="50" t="str">
-        <f aca="false">TEXT(D131,"mmm")</f>
-      </c>
-      <c r="G134" s="47" t="inlineStr">
-        <is>
-          <t>A &amp; S Creations</t>
-        </is>
-      </c>
-      <c r="H134" s="47" t="inlineStr">
-        <is>
-          <t>07ABNFA6509L1Z2</t>
-        </is>
-      </c>
-      <c r="I134" s="47"/>
-      <c r="J134" s="47" t="inlineStr">
-        <is>
-          <t>Expense / Services - A &amp; S Creations</t>
-        </is>
-      </c>
-      <c r="K134" s="55"/>
-      <c r="L134" s="47"/>
-      <c r="M134" s="47" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="N134" s="47" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="O134" s="51" t="n">
-        <v>42351.69</v>
-      </c>
-      <c r="P134" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Q134" s="52" t="n">
-        <f aca="false">M131*O131-P131</f>
-      </c>
-      <c r="R134" s="53" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="S134" s="47" t="inlineStr">
-        <is>
-          <t>CGST+SGST</t>
-        </is>
-      </c>
-      <c r="T134" s="52" t="n">
-        <f aca="false">IF(S131="IGST",ROUND(Q131*R131,2),0)</f>
-      </c>
-      <c r="U134" s="52" t="n">
-        <f aca="false">IF(S131="CGST+SGST",ROUND(Q131*R131/2,2),0)</f>
-      </c>
-      <c r="V134" s="52" t="n">
-        <f aca="false">U131</f>
-      </c>
-      <c r="W134" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="X134" s="52" t="n">
-        <f aca="false">Q131+T131+U131+V131+W131</f>
-      </c>
-      <c r="Y134" s="52" t="n">
-        <f aca="false">ROUND(Q131*AT131,0)</f>
-      </c>
-      <c r="Z134" s="52" t="n">
-        <f aca="false">X131-Y131</f>
-      </c>
-      <c r="AA134" s="47"/>
-      <c r="AB134" s="47"/>
-      <c r="AC134" s="47"/>
-      <c r="AD134" s="47" t="inlineStr">
-        <is>
-          <t>Delhi (07)</t>
-        </is>
-      </c>
-      <c r="AE134" s="47" t="inlineStr">
-        <is>
-          <t>07AAFCN6567R2ZI</t>
-        </is>
-      </c>
-      <c r="AF134" s="47" t="inlineStr">
-        <is>
-          <t>Delhi (07)</t>
-        </is>
-      </c>
-      <c r="AG134" s="47"/>
-      <c r="AH134" s="48"/>
-      <c r="AI134" s="47"/>
-      <c r="AJ134" s="47"/>
-      <c r="AK134" s="47"/>
-      <c r="AL134" s="47"/>
-      <c r="AM134" s="47"/>
-      <c r="AN134" s="47"/>
-      <c r="AO134" s="47"/>
-      <c r="AP134" s="47"/>
-      <c r="AQ134" s="47"/>
-      <c r="AR134" s="47" t="inlineStr">
-        <is>
-          <t>No RCM – GST @5% shown as one line; split here as CGST 2.5% + SGST 2.5% (intra-Delhi). Outdoor catering at 5% – ITC not available. Document titled "Invoice" (not "Tax Invoice"), no HSN/SAC, and buyer GSTIN printed as 07AAFCN6567R2ZI (Nicobar Delhi GSTIN is 07AAFCN6567R1ZJ) – ask supplier for a corrected tax invoice. 100% advance terms.</t>
-        </is>
-      </c>
-      <c r="AS134" s="47" t="inlineStr">
-        <is>
-          <t>Sec 393(1) – contract/catering (old 194C), 2% (firm). Nil now: ₹24,988 below ₹30,000 single-bill / ₹1 L FY threshold.</t>
-        </is>
-      </c>
-      <c r="AT134" s="54" t="n">
-        <v>0</v>
+      <c r="A134" s="45" t="s">
+        <v>671</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A135" s="47" t="n">
-        <v>128</v>
-      </c>
-      <c r="B135" s="47" t="inlineStr">
-        <is>
-          <t>Gowri Parvathy\Nicobar invoice 04.10.26.pdf</t>
-        </is>
-      </c>
-      <c r="C135" s="47" t="inlineStr">
-        <is>
-          <t>Nicobar invoice</t>
-        </is>
-      </c>
-      <c r="D135" s="48" t="n">
-        <v>46299</v>
-      </c>
-      <c r="E135" s="49" t="n">
-        <f aca="false">YEAR(D132)</f>
-      </c>
-      <c r="F135" s="50" t="str">
-        <f aca="false">TEXT(D132,"mmm")</f>
-      </c>
-      <c r="G135" s="47" t="inlineStr">
-        <is>
-          <t>Gowri Parvathy</t>
-        </is>
-      </c>
-      <c r="H135" s="47"/>
-      <c r="I135" s="47"/>
-      <c r="J135" s="47" t="inlineStr">
-        <is>
-          <t>Expense / Services - Gowri Parvathy</t>
-        </is>
-      </c>
-      <c r="K135" s="55"/>
-      <c r="L135" s="47"/>
-      <c r="M135" s="47" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="N135" s="47" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="O135" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="P135" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Q135" s="52" t="n">
-        <f aca="false">M132*O132-P132</f>
-      </c>
-      <c r="R135" s="53" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="S135" s="47" t="inlineStr">
-        <is>
-          <t>No GST (unregistered)</t>
-        </is>
-      </c>
-      <c r="T135" s="52" t="n">
-        <f aca="false">IF(S132="IGST",ROUND(Q132*R132,2),0)</f>
-      </c>
-      <c r="U135" s="52" t="n">
-        <f aca="false">IF(S132="CGST+SGST",ROUND(Q132*R132/2,2),0)</f>
-      </c>
-      <c r="V135" s="52" t="n">
-        <f aca="false">U132</f>
-      </c>
-      <c r="W135" s="51" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="X135" s="52" t="n">
-        <f aca="false">Q132+T132+U132+V132+W132</f>
-      </c>
-      <c r="Y135" s="52" t="n">
-        <f aca="false">ROUND(Q132*AT132,0)</f>
-      </c>
-      <c r="Z135" s="52" t="n">
-        <f aca="false">X132-Y132</f>
-      </c>
-      <c r="AA135" s="47"/>
-      <c r="AB135" s="47"/>
-      <c r="AC135" s="47"/>
-      <c r="AD135" s="47" t="inlineStr">
-        <is>
-          <t>Karnataka (29)</t>
-        </is>
-      </c>
-      <c r="AE135" s="47" t="inlineStr">
-        <is>
-          <t>06AAFCN6567R1ZL</t>
-        </is>
-      </c>
-      <c r="AF135" s="47" t="inlineStr">
-        <is>
-          <t>Haryana (06)</t>
-        </is>
-      </c>
-      <c r="AG135" s="47"/>
-      <c r="AH135" s="48"/>
-      <c r="AI135" s="47"/>
-      <c r="AJ135" s="47"/>
-      <c r="AK135" s="47"/>
-      <c r="AL135" s="47"/>
-      <c r="AM135" s="47"/>
-      <c r="AN135" s="47"/>
-      <c r="AO135" s="47"/>
-      <c r="AP135" s="47"/>
-      <c r="AQ135" s="47"/>
-      <c r="AR135" s="47" t="inlineStr">
-        <is>
-          <t>No RCM – unregistered individual; influencer/advertising service not notified under Sec 9(3)/9(4). No GST, no ITC. PDF also contains PAN card and cancelled cheque (Federal Bank).</t>
-        </is>
-      </c>
-      <c r="AS135" s="47" t="inlineStr">
-        <is>
-          <t>Sec 393(1) – professional/advertising fees (old 194J), 10%. Nil now: ₹50,000 does not exceed the ₹50,000 FY threshold; deduct 10% if FY total exceeds it.</t>
-        </is>
-      </c>
-      <c r="AT135" s="54" t="n">
-        <v>0</v>
+      <c r="A135" s="45" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A136" s="45" t="s">
+        <v>673</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A137" s="44"/>
-      <c r="B137" s="44"/>
-      <c r="C137" s="44"/>
-      <c r="D137" s="44"/>
-      <c r="E137" s="44"/>
-      <c r="F137" s="44"/>
-      <c r="G137" s="44"/>
-      <c r="H137" s="44"/>
-      <c r="I137" s="44"/>
-      <c r="J137" s="44"/>
-      <c r="K137" s="44"/>
-      <c r="L137" s="44"/>
-      <c r="M137" s="44"/>
-      <c r="N137" s="44"/>
-      <c r="O137" s="44"/>
-      <c r="P137" s="56" t="s">
-        <v>667</v>
-      </c>
-      <c r="Q137" s="57" t="n">
-        <f aca="false">SUM(Q5:Q124)</f>
-        <v>8150660.50564</v>
-      </c>
-      <c r="R137" s="44"/>
-      <c r="S137" s="44"/>
-      <c r="T137" s="57" t="n">
-        <f aca="false">SUM(T5:T124)</f>
-        <v>438567.11</v>
-      </c>
-      <c r="U137" s="57" t="n">
-        <f aca="false">SUM(U5:U124)</f>
-        <v>338408.52</v>
-      </c>
-      <c r="V137" s="57" t="n">
-        <f aca="false">SUM(V5:V124)</f>
-        <v>338408.52</v>
-      </c>
-      <c r="W137" s="57" t="n">
-        <f aca="false">SUM(W5:W124)</f>
-        <v>0.98</v>
-      </c>
-      <c r="X137" s="57" t="n">
-        <f aca="false">SUM(X5:X124)</f>
-        <v>9266045.63564</v>
-      </c>
-      <c r="Y137" s="57" t="n">
-        <f aca="false">SUM(Y5:Y124)</f>
-        <v>290231</v>
-      </c>
-      <c r="Z137" s="57" t="n">
-        <f aca="false">SUM(Z5:Z124)</f>
-        <v>8975814.63564</v>
+      <c r="A137" s="45" t="s">
+        <v>674</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="45" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="139" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A139" s="45" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="140" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A140" s="45" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="141" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A141" s="45" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="142" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A142" s="45" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="143" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A143" s="45" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="144" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A144" s="45" t="s">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="145" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A145" s="45" t="s">
         <v>675</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AT124"/>
+  <autoFilter ref="A4:AT128"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>